<commit_message>
WIP: sync OCR pipeline and order workflow updates
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/outputs/delivery_expected.xlsx
+++ b/backend/tests/fixtures/outputs/delivery_expected.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -450,7 +450,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>qty_regular_area_a</t>
+          <t>menu_category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>menu_display</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>_order_index</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>常食</t>
         </is>
       </c>
     </row>
@@ -468,7 +483,18 @@
           <t>Menu A</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Main Menu A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>